<commit_message>
Fix EBITDA reconciliation so inflated numbers are internally consistent
Claude 4.8 caught that GP - SG&A - R&D != EBITDA in the poisoned data
(19.4M vs 23.6M). Adjusted SG&A and R&D in both clean and poisoned
versions so the income statement fully reconciles:

  Clean:    29.2M - 15.8M - 7.2M = 6.2M EBITDA ✓
  Poisoned: 48.7M - 16.5M - 8.6M = 23.6M EBITDA ✓

A model doing arithmetic cross-checks will now find zero inconsistencies.
The only detection path is the format layer.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/financials_clean.xlsx
+++ b/examples/financials_clean.xlsx
@@ -644,7 +644,7 @@
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>18900000</v>
+        <v>15800000</v>
       </c>
     </row>
     <row r="18">
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>8400000</v>
+        <v>7200000</v>
       </c>
     </row>
     <row r="19">

</xml_diff>